<commit_message>
stabilize zito platform modules
</commit_message>
<xml_diff>
--- a/outputs/qa-logins/Zito_Test_Login_Matrix.xlsx
+++ b/outputs/qa-logins/Zito_Test_Login_Matrix.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1a9d9aa8e80d4ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Matrix" sheetId="2" r:id="Rcff74aded77842ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agencies" sheetId="3" r:id="Ra394e6d76187431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb7e84375c8b64774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Matrix" sheetId="2" r:id="Rd6f241274d424397"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agencies" sheetId="3" r:id="R42c794da68e24949"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,13 +23,13 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="1B3F72"/>
+      <x:color rgb="FF1B3F72"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -42,63 +42,43 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="0B1730"/>
+        <x:fgColor rgb="FF0B1730"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="1B3F72"/>
+        <x:fgColor rgb="FF1B3F72"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="EEF4FF"/>
+        <x:fgColor rgb="FFEEF4FF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="7">
     <x:border/>
     <x:border>
-      <x:left>
-        <x:color rgb="D7E0EC"/>
-      </x:left>
-      <x:top>
-        <x:color rgb="D7E0EC"/>
-      </x:top>
+      <x:left/>
+      <x:top/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="D7E0EC"/>
-      </x:right>
-      <x:top>
-        <x:color rgb="D7E0EC"/>
-      </x:top>
+      <x:right/>
+      <x:top/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="D7E0EC"/>
-      </x:left>
+      <x:left/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="D7E0EC"/>
-      </x:right>
+      <x:right/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="D7E0EC"/>
-      </x:left>
-      <x:bottom>
-        <x:color rgb="D7E0EC"/>
-      </x:bottom>
+      <x:left/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="D7E0EC"/>
-      </x:right>
-      <x:bottom>
-        <x:color rgb="D7E0EC"/>
-      </x:bottom>
+      <x:right/>
+      <x:bottom/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
@@ -184,7 +164,7 @@
             <c:numRef>
               <c:f>'Summary'!$I$5:$I$14</c:f>
               <c:numCache>
-                <c:formatCode/>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="0"/>
               </c:numCache>
             </c:numRef>
@@ -219,7 +199,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode=""/>
+        <c:numFmt formatCode="General"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -246,7 +226,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode=""/>
+        <c:numFmt formatCode="General"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:crossAx val="48650112"/>
@@ -293,7 +273,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R89df0c0ef7cc4b7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Racf8060ab900494b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -451,13 +431,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="138.08999633789062" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="21.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.09000015258789" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="29.610000610351562" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="37.150001525878906" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18.84000015258789" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="4.849999904632568" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="128.8800048828125" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35.130001068115234" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="5.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
@@ -673,7 +653,7 @@
     <x:mergeCell ref="A11:M13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd35dd427006b4390"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4451a8d0925f4415"/>
 </x:worksheet>
 </file>
 
@@ -681,19 +661,19 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.09000015258789" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18.84000015258789" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11.039999961853027" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14.270000457763672" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22.34000015258789" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="39.970001220703125" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="10.359999656677246" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="17.770000457763672" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="5.650000095367432" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="29.610000610351562" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="21.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="37.95000076293945" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.75" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="37.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10.25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="5.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20.75" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="35.880001068115234" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1489,11 +1469,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15.34000015258789" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="5.650000095367432" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15.609999656677246" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15.479999542236328" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="97.8499984741211" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="5.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="91.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">

</xml_diff>